<commit_message>
fix(bc-tmfn): knockout rounds count back from the final, as the EKC sheets print
The 34th EKC 2026 Junior Individual Male sheet (page 4, court A) prints
P2 v P3 alone in column 1 and P4 v P5 beside P1 v Winner F1 in column 2;
the 33rd EKC 2025 Men Team five-team courts, and the 2026 Junior
Individual Female and Men Individual sheets, print the same way. An
earlier reading put P4 v P5 in column 1 and pulled every pair beside an
empty pair forward a round (the "risen" classification), so a
five-player knockout showed its semifinal pair as a quarterfinal.

A bout's round is now its distance from the final on every surface: the
app bracket, match numbers, order of play, and the Excel columns. The
pairings are unchanged; the rise marks stay as slot geometry only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knockout-example-large-seeded.xlsx
+++ b/knockout-example-large-seeded.xlsx
@@ -959,175 +959,175 @@
     <t>2.</t>
   </si>
   <si>
+    <t>Round 1 - Match 14</t>
+  </si>
+  <si>
+    <t>Round 1 - Match 2</t>
+  </si>
+  <si>
+    <t>Round 1 - Match 15</t>
+  </si>
+  <si>
+    <t>Round 1 - Match 3</t>
+  </si>
+  <si>
+    <t>Round 1 - Match 16</t>
+  </si>
+  <si>
+    <t>Round 1 - Match 4</t>
+  </si>
+  <si>
     <t>Round 1 - Match 17</t>
   </si>
   <si>
-    <t>Round 1 - Match 2</t>
+    <t>Round 1 - Match 5</t>
   </si>
   <si>
     <t>Round 1 - Match 18</t>
   </si>
   <si>
-    <t>Round 1 - Match 3</t>
+    <t>Round 1 - Match 6</t>
   </si>
   <si>
     <t>Round 1 - Match 19</t>
   </si>
   <si>
-    <t>Round 1 - Match 4</t>
+    <t>Round 1 - Match 7</t>
   </si>
   <si>
     <t>Round 1 - Match 20</t>
   </si>
   <si>
-    <t>Round 1 - Match 5</t>
+    <t>Round 1 - Match 8</t>
   </si>
   <si>
     <t>Round 1 - Match 21</t>
   </si>
   <si>
-    <t>Round 1 - Match 6</t>
+    <t>Round 1 - Match 9</t>
   </si>
   <si>
     <t>Round 1 - Match 22</t>
   </si>
   <si>
-    <t>Round 1 - Match 7</t>
+    <t>Round 1 - Match 10</t>
   </si>
   <si>
     <t>Round 1 - Match 23</t>
   </si>
   <si>
-    <t>Round 1 - Match 8</t>
+    <t>Round 1 - Match 11</t>
   </si>
   <si>
     <t>Round 1 - Match 24</t>
   </si>
   <si>
-    <t>Round 1 - Match 9</t>
+    <t>Round 1 - Match 12</t>
   </si>
   <si>
     <t>Round 1 - Match 25</t>
   </si>
   <si>
-    <t>Round 1 - Match 10</t>
+    <t>Round 1 - Match 13</t>
   </si>
   <si>
     <t>Round 1 - Match 26</t>
   </si>
   <si>
-    <t>Round 1 - Match 11</t>
-  </si>
-  <si>
     <t>Round 1 - Match 27</t>
   </si>
   <si>
-    <t>Round 1 - Match 12</t>
-  </si>
-  <si>
-    <t>Round 1 - Match 28</t>
-  </si>
-  <si>
-    <t>Round 1 - Match 13</t>
-  </si>
-  <si>
-    <t>Round 1 - Match 29</t>
-  </si>
-  <si>
-    <t>Round 1 - Match 14</t>
-  </si>
-  <si>
-    <t>Round 1 - Match 30</t>
-  </si>
-  <si>
-    <t>Round 1 - Match 15</t>
-  </si>
-  <si>
-    <t>Round 1 - Match 31</t>
-  </si>
-  <si>
-    <t>Round 1 - Match 16</t>
-  </si>
-  <si>
-    <t>Round 1 - Match 32</t>
+    <t>Round 2 - Match 28</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 44</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 29</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 45</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 30</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 46</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 31</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 47</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 32</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 48</t>
   </si>
   <si>
     <t>Round 2 - Match 33</t>
   </si>
   <si>
-    <t>Round 2 - Match 46</t>
+    <t>Round 2 - Match 49</t>
   </si>
   <si>
     <t>Round 2 - Match 34</t>
   </si>
   <si>
-    <t>Round 2 - Match 47</t>
+    <t>Round 2 - Match 50</t>
   </si>
   <si>
     <t>Round 2 - Match 35</t>
   </si>
   <si>
-    <t>Round 2 - Match 48</t>
+    <t>Round 2 - Match 51</t>
   </si>
   <si>
     <t>Round 2 - Match 36</t>
   </si>
   <si>
-    <t>Round 2 - Match 49</t>
+    <t>Round 2 - Match 52</t>
   </si>
   <si>
     <t>Round 2 - Match 37</t>
   </si>
   <si>
-    <t>Round 2 - Match 50</t>
+    <t>Round 2 - Match 53</t>
   </si>
   <si>
     <t>Round 2 - Match 38</t>
   </si>
   <si>
-    <t>Round 2 - Match 51</t>
+    <t>Round 2 - Match 54</t>
   </si>
   <si>
     <t>Round 2 - Match 39</t>
   </si>
   <si>
-    <t>Round 2 - Match 52</t>
+    <t>Round 2 - Match 55</t>
   </si>
   <si>
     <t>Round 2 - Match 40</t>
   </si>
   <si>
-    <t>Round 2 - Match 53</t>
+    <t>Round 2 - Match 56</t>
   </si>
   <si>
     <t>Round 2 - Match 41</t>
   </si>
   <si>
-    <t>Round 2 - Match 54</t>
+    <t>Round 2 - Match 57</t>
   </si>
   <si>
     <t>Round 2 - Match 42</t>
   </si>
   <si>
-    <t>Round 2 - Match 55</t>
+    <t>Round 2 - Match 58</t>
   </si>
   <si>
     <t>Round 2 - Match 43</t>
-  </si>
-  <si>
-    <t>Round 2 - Match 56</t>
-  </si>
-  <si>
-    <t>Round 2 - Match 44</t>
-  </si>
-  <si>
-    <t>Round 2 - Match 57</t>
-  </si>
-  <si>
-    <t>Round 2 - Match 45</t>
-  </si>
-  <si>
-    <t>Round 2 - Match 58</t>
   </si>
   <si>
     <t>Round 2 - Match 59</t>
@@ -3388,29 +3388,35 @@
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
     </row>
-    <row r="5">
-      <c r="C5" s="16" t="s">
+    <row r="6">
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="6">
-      <c r="D6" s="14"/>
-      <c r="E6" s="13">
-        <v>9</v>
-      </c>
-    </row>
     <row r="7">
-      <c r="C7" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="12"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="12"/>
+    </row>
+    <row r="8">
+      <c r="G8" s="13">
+        <v>36</v>
+      </c>
     </row>
     <row r="9">
+      <c r="G9" s="12"/>
       <c r="H9" s="14"/>
       <c r="I9" s="12"/>
     </row>
     <row r="10">
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="F10" s="15"/>
+      <c r="G10" s="12"/>
       <c r="I10" s="12"/>
     </row>
     <row r="11">
@@ -3443,7 +3449,7 @@
     </row>
     <row r="16">
       <c r="G16" s="13">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H16" s="15"/>
       <c r="I16" s="12"/>
@@ -3459,7 +3465,7 @@
     <row r="18">
       <c r="D18" s="14"/>
       <c r="E18" s="13">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F18" s="15"/>
       <c r="G18" s="12"/>
@@ -3496,7 +3502,7 @@
     </row>
     <row r="24">
       <c r="G24" s="13">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="K24" s="12"/>
     </row>
@@ -3512,7 +3518,7 @@
     <row r="26">
       <c r="D26" s="14"/>
       <c r="E26" s="13">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F26" s="15"/>
       <c r="G26" s="12"/>
@@ -3553,7 +3559,7 @@
     </row>
     <row r="32">
       <c r="G32" s="13">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="H32" s="15"/>
       <c r="I32" s="12"/>
@@ -3567,7 +3573,7 @@
     <row r="34">
       <c r="D34" s="14"/>
       <c r="E34" s="13">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F34" s="15"/>
       <c r="G34" s="12"/>
@@ -3631,7 +3637,7 @@
     </row>
     <row r="8">
       <c r="G8" s="13">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9">
@@ -3645,7 +3651,7 @@
     <row r="10">
       <c r="D10" s="14"/>
       <c r="E10" s="13">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F10" s="15"/>
       <c r="G10" s="12"/>
@@ -3686,7 +3692,7 @@
     </row>
     <row r="16">
       <c r="G16" s="13">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="H16" s="15"/>
       <c r="I16" s="12"/>
@@ -3702,7 +3708,7 @@
     <row r="18">
       <c r="D18" s="14"/>
       <c r="E18" s="13">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F18" s="15"/>
       <c r="G18" s="12"/>
@@ -3739,7 +3745,7 @@
     </row>
     <row r="24">
       <c r="G24" s="13">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="K24" s="12"/>
     </row>
@@ -3755,7 +3761,7 @@
     <row r="26">
       <c r="D26" s="14"/>
       <c r="E26" s="13">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F26" s="15"/>
       <c r="G26" s="12"/>
@@ -3796,7 +3802,7 @@
     </row>
     <row r="32">
       <c r="G32" s="13">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="H32" s="15"/>
       <c r="I32" s="12"/>
@@ -3810,7 +3816,7 @@
     <row r="34">
       <c r="D34" s="14"/>
       <c r="E34" s="13">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F34" s="15"/>
       <c r="G34" s="12"/>
@@ -3861,29 +3867,35 @@
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
     </row>
-    <row r="5">
-      <c r="C5" s="16" t="s">
+    <row r="6">
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="6">
-      <c r="D6" s="14"/>
-      <c r="E6" s="13">
-        <v>17</v>
-      </c>
-    </row>
     <row r="7">
-      <c r="C7" s="16" t="s">
-        <v>178</v>
-      </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="12"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="12"/>
+    </row>
+    <row r="8">
+      <c r="G8" s="13">
+        <v>44</v>
+      </c>
     </row>
     <row r="9">
+      <c r="G9" s="12"/>
       <c r="H9" s="14"/>
       <c r="I9" s="12"/>
     </row>
     <row r="10">
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="F10" s="15"/>
+      <c r="G10" s="12"/>
       <c r="I10" s="12"/>
     </row>
     <row r="11">
@@ -3916,7 +3928,7 @@
     </row>
     <row r="16">
       <c r="G16" s="13">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H16" s="15"/>
       <c r="I16" s="12"/>
@@ -3932,7 +3944,7 @@
     <row r="18">
       <c r="D18" s="14"/>
       <c r="E18" s="13">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F18" s="15"/>
       <c r="G18" s="12"/>
@@ -3969,7 +3981,7 @@
     </row>
     <row r="24">
       <c r="G24" s="13">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K24" s="12"/>
     </row>
@@ -3985,7 +3997,7 @@
     <row r="26">
       <c r="D26" s="14"/>
       <c r="E26" s="13">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F26" s="15"/>
       <c r="G26" s="12"/>
@@ -4026,7 +4038,7 @@
     </row>
     <row r="32">
       <c r="G32" s="13">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H32" s="15"/>
       <c r="I32" s="12"/>
@@ -4040,7 +4052,7 @@
     <row r="34">
       <c r="D34" s="14"/>
       <c r="E34" s="13">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F34" s="15"/>
       <c r="G34" s="12"/>
@@ -4104,7 +4116,7 @@
     </row>
     <row r="8">
       <c r="G8" s="13">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9">
@@ -4118,7 +4130,7 @@
     <row r="10">
       <c r="D10" s="14"/>
       <c r="E10" s="13">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F10" s="15"/>
       <c r="G10" s="12"/>
@@ -4159,7 +4171,7 @@
     </row>
     <row r="16">
       <c r="G16" s="13">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H16" s="15"/>
       <c r="I16" s="12"/>
@@ -4175,7 +4187,7 @@
     <row r="18">
       <c r="D18" s="14"/>
       <c r="E18" s="13">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F18" s="15"/>
       <c r="G18" s="12"/>
@@ -4212,7 +4224,7 @@
     </row>
     <row r="24">
       <c r="G24" s="13">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K24" s="12"/>
     </row>
@@ -4228,7 +4240,7 @@
     <row r="26">
       <c r="D26" s="14"/>
       <c r="E26" s="13">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F26" s="15"/>
       <c r="G26" s="12"/>
@@ -4269,7 +4281,7 @@
     </row>
     <row r="32">
       <c r="G32" s="13">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H32" s="15"/>
       <c r="I32" s="12"/>
@@ -4283,7 +4295,7 @@
     <row r="34">
       <c r="D34" s="14"/>
       <c r="E34" s="13">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F34" s="15"/>
       <c r="G34" s="12"/>
@@ -4334,29 +4346,35 @@
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
     </row>
-    <row r="5">
-      <c r="C5" s="16" t="s">
+    <row r="6">
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="6">
-      <c r="D6" s="14"/>
-      <c r="E6" s="13">
-        <v>25</v>
-      </c>
-    </row>
     <row r="7">
-      <c r="C7" s="16" t="s">
-        <v>241</v>
-      </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="12"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="12"/>
+    </row>
+    <row r="8">
+      <c r="G8" s="13">
+        <v>52</v>
+      </c>
     </row>
     <row r="9">
+      <c r="G9" s="12"/>
       <c r="H9" s="14"/>
       <c r="I9" s="12"/>
     </row>
     <row r="10">
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16" t="s">
+        <v>241</v>
+      </c>
+      <c r="F10" s="15"/>
+      <c r="G10" s="12"/>
       <c r="I10" s="12"/>
     </row>
     <row r="11">
@@ -4405,7 +4423,7 @@
     <row r="18">
       <c r="D18" s="14"/>
       <c r="E18" s="13">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F18" s="15"/>
       <c r="G18" s="12"/>
@@ -4458,7 +4476,7 @@
     <row r="26">
       <c r="D26" s="14"/>
       <c r="E26" s="13">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F26" s="15"/>
       <c r="G26" s="12"/>
@@ -4513,7 +4531,7 @@
     <row r="34">
       <c r="D34" s="14"/>
       <c r="E34" s="13">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F34" s="15"/>
       <c r="G34" s="12"/>
@@ -4591,7 +4609,7 @@
     <row r="10">
       <c r="D10" s="14"/>
       <c r="E10" s="13">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F10" s="15"/>
       <c r="G10" s="12"/>
@@ -4648,7 +4666,7 @@
     <row r="18">
       <c r="D18" s="14"/>
       <c r="E18" s="13">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F18" s="15"/>
       <c r="G18" s="12"/>
@@ -4701,7 +4719,7 @@
     <row r="26">
       <c r="D26" s="14"/>
       <c r="E26" s="13">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F26" s="15"/>
       <c r="G26" s="12"/>
@@ -4756,7 +4774,7 @@
     <row r="34">
       <c r="D34" s="14"/>
       <c r="E34" s="13">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="F34" s="15"/>
       <c r="G34" s="12"/>
@@ -5929,7 +5947,7 @@
     </row>
     <row r="4">
       <c r="A4" s="19" t="str">
-        <f>'data'!$B$4</f>
+        <f>'data'!$B$80</f>
       </c>
       <c r="B4" s="22"/>
       <c r="C4" s="22"/>
@@ -5937,10 +5955,10 @@
       <c r="E4" s="22"/>
       <c r="F4" s="22"/>
       <c r="G4" s="19" t="str">
-        <f>'data'!$B$60</f>
+        <f>'data'!$B$6</f>
       </c>
       <c r="I4" s="19" t="str">
-        <f>'data'!$B$49</f>
+        <f>'data'!$B$52</f>
       </c>
       <c r="J4" s="22"/>
       <c r="K4" s="22"/>
@@ -5948,7 +5966,7 @@
       <c r="M4" s="22"/>
       <c r="N4" s="22"/>
       <c r="O4" s="19" t="str">
-        <f>'data'!$B$48</f>
+        <f>'data'!$B$51</f>
       </c>
     </row>
     <row r="6">
@@ -6013,7 +6031,7 @@
     </row>
     <row r="12">
       <c r="A12" s="19" t="str">
-        <f>'data'!$B$80</f>
+        <f>'data'!$B$10</f>
       </c>
       <c r="B12" s="22"/>
       <c r="C12" s="22"/>
@@ -6021,10 +6039,10 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
       <c r="G12" s="19" t="str">
-        <f>'data'!$B$6</f>
+        <f>'data'!$B$87</f>
       </c>
       <c r="I12" s="19" t="str">
-        <f>'data'!$B$52</f>
+        <f>'data'!$B$55</f>
       </c>
       <c r="J12" s="22"/>
       <c r="K12" s="22"/>
@@ -6032,7 +6050,7 @@
       <c r="M12" s="22"/>
       <c r="N12" s="22"/>
       <c r="O12" s="19" t="str">
-        <f>'data'!$B$51</f>
+        <f>'data'!$B$54</f>
       </c>
     </row>
     <row r="14">
@@ -6097,7 +6115,7 @@
     </row>
     <row r="20">
       <c r="A20" s="19" t="str">
-        <f>'data'!$B$10</f>
+        <f>'data'!$B$13</f>
       </c>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -6105,10 +6123,10 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
       <c r="G20" s="19" t="str">
-        <f>'data'!$B$87</f>
+        <f>'data'!$B$90</f>
       </c>
       <c r="I20" s="19" t="str">
-        <f>'data'!$B$55</f>
+        <f>'data'!$B$58</f>
       </c>
       <c r="J20" s="22"/>
       <c r="K20" s="22"/>
@@ -6116,7 +6134,7 @@
       <c r="M20" s="22"/>
       <c r="N20" s="22"/>
       <c r="O20" s="19" t="str">
-        <f>'data'!$B$54</f>
+        <f>'data'!$B$57</f>
       </c>
     </row>
     <row r="22">
@@ -6181,7 +6199,7 @@
     </row>
     <row r="28">
       <c r="A28" s="19" t="str">
-        <f>'data'!$B$13</f>
+        <f>'data'!$B$18</f>
       </c>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -6189,10 +6207,10 @@
       <c r="E28" s="22"/>
       <c r="F28" s="22"/>
       <c r="G28" s="19" t="str">
-        <f>'data'!$B$90</f>
+        <f>'data'!$B$17</f>
       </c>
       <c r="I28" s="19" t="str">
-        <f>'data'!$B$58</f>
+        <f>'data'!$B$61</f>
       </c>
       <c r="J28" s="22"/>
       <c r="K28" s="22"/>
@@ -6200,7 +6218,7 @@
       <c r="M28" s="22"/>
       <c r="N28" s="22"/>
       <c r="O28" s="19" t="str">
-        <f>'data'!$B$57</f>
+        <f>'data'!$B$60</f>
       </c>
     </row>
     <row r="30">
@@ -6265,7 +6283,7 @@
     </row>
     <row r="36">
       <c r="A36" s="19" t="str">
-        <f>'data'!$B$15</f>
+        <f>'data'!$B$21</f>
       </c>
       <c r="B36" s="22"/>
       <c r="C36" s="22"/>
@@ -6273,10 +6291,10 @@
       <c r="E36" s="22"/>
       <c r="F36" s="22"/>
       <c r="G36" s="19" t="str">
-        <f>'data'!$B$14</f>
+        <f>'data'!$B$20</f>
       </c>
       <c r="I36" s="19" t="str">
-        <f>'data'!$B$61</f>
+        <f>'data'!$B$64</f>
       </c>
       <c r="J36" s="22"/>
       <c r="K36" s="22"/>
@@ -6284,7 +6302,7 @@
       <c r="M36" s="22"/>
       <c r="N36" s="22"/>
       <c r="O36" s="19" t="str">
-        <f>'data'!$B$60</f>
+        <f>'data'!$B$63</f>
       </c>
     </row>
     <row r="38">
@@ -6349,7 +6367,7 @@
     </row>
     <row r="44">
       <c r="A44" s="19" t="str">
-        <f>'data'!$B$18</f>
+        <f>'data'!$B$24</f>
       </c>
       <c r="B44" s="22"/>
       <c r="C44" s="22"/>
@@ -6357,10 +6375,10 @@
       <c r="E44" s="22"/>
       <c r="F44" s="22"/>
       <c r="G44" s="19" t="str">
-        <f>'data'!$B$17</f>
+        <f>'data'!$B$23</f>
       </c>
       <c r="I44" s="19" t="str">
-        <f>'data'!$B$64</f>
+        <f>'data'!$B$67</f>
       </c>
       <c r="J44" s="22"/>
       <c r="K44" s="22"/>
@@ -6368,7 +6386,7 @@
       <c r="M44" s="22"/>
       <c r="N44" s="22"/>
       <c r="O44" s="19" t="str">
-        <f>'data'!$B$63</f>
+        <f>'data'!$B$66</f>
       </c>
     </row>
     <row r="46">
@@ -6433,7 +6451,7 @@
     </row>
     <row r="52">
       <c r="A52" s="19" t="str">
-        <f>'data'!$B$21</f>
+        <f>'data'!$B$29</f>
       </c>
       <c r="B52" s="22"/>
       <c r="C52" s="22"/>
@@ -6441,10 +6459,10 @@
       <c r="E52" s="22"/>
       <c r="F52" s="22"/>
       <c r="G52" s="19" t="str">
-        <f>'data'!$B$20</f>
+        <f>'data'!$B$28</f>
       </c>
       <c r="I52" s="19" t="str">
-        <f>'data'!$B$67</f>
+        <f>'data'!$B$70</f>
       </c>
       <c r="J52" s="22"/>
       <c r="K52" s="22"/>
@@ -6452,7 +6470,7 @@
       <c r="M52" s="22"/>
       <c r="N52" s="22"/>
       <c r="O52" s="19" t="str">
-        <f>'data'!$B$66</f>
+        <f>'data'!$B$73</f>
       </c>
     </row>
     <row r="54">
@@ -6517,7 +6535,7 @@
     </row>
     <row r="60">
       <c r="A60" s="19" t="str">
-        <f>'data'!$B$24</f>
+        <f>'data'!$B$55</f>
       </c>
       <c r="B60" s="22"/>
       <c r="C60" s="22"/>
@@ -6525,10 +6543,10 @@
       <c r="E60" s="22"/>
       <c r="F60" s="22"/>
       <c r="G60" s="19" t="str">
-        <f>'data'!$B$23</f>
+        <f>'data'!$B$31</f>
       </c>
       <c r="I60" s="19" t="str">
-        <f>'data'!$B$70</f>
+        <f>'data'!$B$75</f>
       </c>
       <c r="J60" s="22"/>
       <c r="K60" s="22"/>
@@ -6536,7 +6554,7 @@
       <c r="M60" s="22"/>
       <c r="N60" s="22"/>
       <c r="O60" s="19" t="str">
-        <f>'data'!$B$73</f>
+        <f>'data'!$B$74</f>
       </c>
     </row>
     <row r="62">
@@ -6601,7 +6619,7 @@
     </row>
     <row r="68">
       <c r="A68" s="19" t="str">
-        <f>'data'!$B$26</f>
+        <f>'data'!$B$35</f>
       </c>
       <c r="B68" s="22"/>
       <c r="C68" s="22"/>
@@ -6609,10 +6627,10 @@
       <c r="E68" s="22"/>
       <c r="F68" s="22"/>
       <c r="G68" s="19" t="str">
-        <f>'data'!$B$25</f>
+        <f>'data'!$B$56</f>
       </c>
       <c r="I68" s="19" t="str">
-        <f>'data'!$B$72</f>
+        <f>'data'!$B$78</f>
       </c>
       <c r="J68" s="22"/>
       <c r="K68" s="22"/>
@@ -6620,7 +6638,7 @@
       <c r="M68" s="22"/>
       <c r="N68" s="22"/>
       <c r="O68" s="19" t="str">
-        <f>'data'!$B$71</f>
+        <f>'data'!$B$77</f>
       </c>
     </row>
     <row r="70">
@@ -6685,7 +6703,7 @@
     </row>
     <row r="76">
       <c r="A76" s="19" t="str">
-        <f>'data'!$B$29</f>
+        <f>'data'!$B$70</f>
       </c>
       <c r="B76" s="22"/>
       <c r="C76" s="22"/>
@@ -6693,10 +6711,10 @@
       <c r="E76" s="22"/>
       <c r="F76" s="22"/>
       <c r="G76" s="19" t="str">
-        <f>'data'!$B$28</f>
+        <f>'data'!$B$53</f>
       </c>
       <c r="I76" s="19" t="str">
-        <f>'data'!$B$75</f>
+        <f>'data'!$B$81</f>
       </c>
       <c r="J76" s="22"/>
       <c r="K76" s="22"/>
@@ -6704,7 +6722,7 @@
       <c r="M76" s="22"/>
       <c r="N76" s="22"/>
       <c r="O76" s="19" t="str">
-        <f>'data'!$B$74</f>
+        <f>'data'!$B$80</f>
       </c>
     </row>
     <row r="78">
@@ -6769,7 +6787,7 @@
     </row>
     <row r="84">
       <c r="A84" s="19" t="str">
-        <f>'data'!$B$55</f>
+        <f>'data'!$B$41</f>
       </c>
       <c r="B84" s="22"/>
       <c r="C84" s="22"/>
@@ -6777,10 +6795,10 @@
       <c r="E84" s="22"/>
       <c r="F84" s="22"/>
       <c r="G84" s="19" t="str">
-        <f>'data'!$B$31</f>
+        <f>'data'!$B$40</f>
       </c>
       <c r="I84" s="19" t="str">
-        <f>'data'!$B$78</f>
+        <f>'data'!$B$93</f>
       </c>
       <c r="J84" s="22"/>
       <c r="K84" s="22"/>
@@ -6788,7 +6806,7 @@
       <c r="M84" s="22"/>
       <c r="N84" s="22"/>
       <c r="O84" s="19" t="str">
-        <f>'data'!$B$77</f>
+        <f>'data'!$B$83</f>
       </c>
     </row>
     <row r="86">
@@ -6853,7 +6871,7 @@
     </row>
     <row r="92">
       <c r="A92" s="19" t="str">
-        <f>'data'!$B$35</f>
+        <f>'data'!$B$44</f>
       </c>
       <c r="B92" s="22"/>
       <c r="C92" s="22"/>
@@ -6861,10 +6879,10 @@
       <c r="E92" s="22"/>
       <c r="F92" s="22"/>
       <c r="G92" s="19" t="str">
-        <f>'data'!$B$56</f>
+        <f>'data'!$B$43</f>
       </c>
       <c r="I92" s="19" t="str">
-        <f>'data'!$B$81</f>
+        <f>'data'!$B$87</f>
       </c>
       <c r="J92" s="22"/>
       <c r="K92" s="22"/>
@@ -6872,7 +6890,7 @@
       <c r="M92" s="22"/>
       <c r="N92" s="22"/>
       <c r="O92" s="19" t="str">
-        <f>'data'!$B$80</f>
+        <f>'data'!$B$86</f>
       </c>
     </row>
     <row r="94">
@@ -6937,7 +6955,7 @@
     </row>
     <row r="100">
       <c r="A100" s="19" t="str">
-        <f>'data'!$B$70</f>
+        <f>'data'!$B$47</f>
       </c>
       <c r="B100" s="22"/>
       <c r="C100" s="22"/>
@@ -6945,10 +6963,10 @@
       <c r="E100" s="22"/>
       <c r="F100" s="22"/>
       <c r="G100" s="19" t="str">
-        <f>'data'!$B$53</f>
+        <f>'data'!$B$46</f>
       </c>
       <c r="I100" s="19" t="str">
-        <f>'data'!$B$93</f>
+        <f>'data'!$B$90</f>
       </c>
       <c r="J100" s="22"/>
       <c r="K100" s="22"/>
@@ -6956,7 +6974,7 @@
       <c r="M100" s="22"/>
       <c r="N100" s="22"/>
       <c r="O100" s="19" t="str">
-        <f>'data'!$B$83</f>
+        <f>'data'!$B$89</f>
       </c>
     </row>
     <row r="102">
@@ -6980,17 +6998,8 @@
       <c r="O103" s="23"/>
     </row>
     <row r="106">
-      <c r="A106" s="11" t="s">
+      <c r="I106" s="11" t="s">
         <v>331</v>
-      </c>
-      <c r="B106" s="11"/>
-      <c r="C106" s="11"/>
-      <c r="D106" s="11"/>
-      <c r="E106" s="11"/>
-      <c r="F106" s="11"/>
-      <c r="G106" s="11"/>
-      <c r="I106" s="11" t="s">
-        <v>332</v>
       </c>
       <c r="J106" s="11"/>
       <c r="K106" s="11"/>
@@ -7000,15 +7009,6 @@
       <c r="O106" s="11"/>
     </row>
     <row r="107">
-      <c r="A107" s="21" t="s">
-        <v>301</v>
-      </c>
-      <c r="D107" s="19" t="s">
-        <v>302</v>
-      </c>
-      <c r="G107" s="20" t="s">
-        <v>303</v>
-      </c>
       <c r="I107" s="21" t="s">
         <v>301</v>
       </c>
@@ -7020,19 +7020,8 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="19" t="str">
-        <f>'data'!$B$41</f>
-      </c>
-      <c r="B108" s="22"/>
-      <c r="C108" s="22"/>
-      <c r="D108" s="22"/>
-      <c r="E108" s="22"/>
-      <c r="F108" s="22"/>
-      <c r="G108" s="19" t="str">
-        <f>'data'!$B$40</f>
-      </c>
       <c r="I108" s="19" t="str">
-        <f>'data'!$B$87</f>
+        <f>'data'!$B$93</f>
       </c>
       <c r="J108" s="22"/>
       <c r="K108" s="22"/>
@@ -7040,200 +7029,192 @@
       <c r="M108" s="22"/>
       <c r="N108" s="22"/>
       <c r="O108" s="19" t="str">
-        <f>'data'!$B$86</f>
+        <f>'data'!$B$92</f>
       </c>
     </row>
     <row r="110">
-      <c r="F110" t="s">
-        <v>304</v>
-      </c>
-      <c r="G110" s="23"/>
       <c r="N110" t="s">
         <v>304</v>
       </c>
       <c r="O110" s="23"/>
     </row>
     <row r="111">
-      <c r="F111" t="s">
-        <v>305</v>
-      </c>
-      <c r="G111" s="23"/>
       <c r="N111" t="s">
         <v>305</v>
       </c>
       <c r="O111" s="23"/>
     </row>
-    <row r="114">
-      <c r="A114" s="11" t="s">
+    <row r="119">
+      <c r="A119" s="11" t="s">
+        <v>332</v>
+      </c>
+      <c r="B119" s="11"/>
+      <c r="C119" s="11"/>
+      <c r="D119" s="11"/>
+      <c r="E119" s="11"/>
+      <c r="F119" s="11"/>
+      <c r="G119" s="11"/>
+      <c r="I119" s="11" t="s">
         <v>333</v>
       </c>
-      <c r="B114" s="11"/>
-      <c r="C114" s="11"/>
-      <c r="D114" s="11"/>
-      <c r="E114" s="11"/>
-      <c r="F114" s="11"/>
-      <c r="G114" s="11"/>
-      <c r="I114" s="11" t="s">
+      <c r="J119" s="11"/>
+      <c r="K119" s="11"/>
+      <c r="L119" s="11"/>
+      <c r="M119" s="11"/>
+      <c r="N119" s="11"/>
+      <c r="O119" s="11"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="21" t="s">
+        <v>301</v>
+      </c>
+      <c r="D120" s="19" t="s">
+        <v>302</v>
+      </c>
+      <c r="G120" s="20" t="s">
+        <v>303</v>
+      </c>
+      <c r="I120" s="21" t="s">
+        <v>301</v>
+      </c>
+      <c r="L120" s="19" t="s">
+        <v>302</v>
+      </c>
+      <c r="O120" s="20" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="19" t="str">
+        <f>'data'!$B$4</f>
+      </c>
+      <c r="B121" s="22"/>
+      <c r="C121" s="22"/>
+      <c r="D121" s="22"/>
+      <c r="E121" s="22"/>
+      <c r="F121" s="22"/>
+      <c r="G121" s="19" t="str">
+        <f>'data'!$B$60</f>
+      </c>
+      <c r="I121" s="19" t="str">
+        <f>'data'!$B$49</f>
+      </c>
+      <c r="J121" s="22"/>
+      <c r="K121" s="22"/>
+      <c r="L121" s="22"/>
+      <c r="M121" s="22"/>
+      <c r="N121" s="22"/>
+      <c r="O121" s="19" t="str">
+        <f>'data'!$B$48</f>
+      </c>
+    </row>
+    <row r="123">
+      <c r="F123" t="s">
+        <v>304</v>
+      </c>
+      <c r="G123" s="23"/>
+      <c r="N123" t="s">
+        <v>304</v>
+      </c>
+      <c r="O123" s="23"/>
+    </row>
+    <row r="124">
+      <c r="F124" t="s">
+        <v>305</v>
+      </c>
+      <c r="G124" s="23"/>
+      <c r="N124" t="s">
+        <v>305</v>
+      </c>
+      <c r="O124" s="23"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="11" t="s">
         <v>334</v>
       </c>
-      <c r="J114" s="11"/>
-      <c r="K114" s="11"/>
-      <c r="L114" s="11"/>
-      <c r="M114" s="11"/>
-      <c r="N114" s="11"/>
-      <c r="O114" s="11"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="21" t="s">
+      <c r="B127" s="11"/>
+      <c r="C127" s="11"/>
+      <c r="D127" s="11"/>
+      <c r="E127" s="11"/>
+      <c r="F127" s="11"/>
+      <c r="G127" s="11"/>
+      <c r="I127" s="11" t="s">
+        <v>335</v>
+      </c>
+      <c r="J127" s="11"/>
+      <c r="K127" s="11"/>
+      <c r="L127" s="11"/>
+      <c r="M127" s="11"/>
+      <c r="N127" s="11"/>
+      <c r="O127" s="11"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="21" t="s">
         <v>301</v>
       </c>
-      <c r="D115" s="19" t="s">
+      <c r="D128" s="19" t="s">
         <v>302</v>
       </c>
-      <c r="G115" s="20" t="s">
+      <c r="G128" s="20" t="s">
         <v>303</v>
       </c>
-      <c r="I115" s="21" t="s">
+      <c r="I128" s="21" t="s">
         <v>301</v>
       </c>
-      <c r="L115" s="19" t="s">
+      <c r="L128" s="19" t="s">
         <v>302</v>
       </c>
-      <c r="O115" s="20" t="s">
+      <c r="O128" s="20" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" s="19" t="str">
-        <f>'data'!$B$44</f>
-      </c>
-      <c r="B116" s="22"/>
-      <c r="C116" s="22"/>
-      <c r="D116" s="22"/>
-      <c r="E116" s="22"/>
-      <c r="F116" s="22"/>
-      <c r="G116" s="19" t="str">
-        <f>'data'!$B$43</f>
-      </c>
-      <c r="I116" s="19" t="str">
-        <f>'data'!$B$90</f>
-      </c>
-      <c r="J116" s="22"/>
-      <c r="K116" s="22"/>
-      <c r="L116" s="22"/>
-      <c r="M116" s="22"/>
-      <c r="N116" s="22"/>
-      <c r="O116" s="19" t="str">
-        <f>'data'!$B$89</f>
-      </c>
-    </row>
-    <row r="118">
-      <c r="F118" t="s">
+    <row r="129">
+      <c r="A129" s="19" t="str">
+        <f>CONCATENATE("M 1 ",G6)</f>
+      </c>
+      <c r="B129" s="22"/>
+      <c r="C129" s="22"/>
+      <c r="D129" s="22"/>
+      <c r="E129" s="22"/>
+      <c r="F129" s="22"/>
+      <c r="G129" s="19" t="str">
+        <f>'data'!$B$5</f>
+      </c>
+      <c r="I129" s="19" t="str">
+        <f>CONCATENATE("M 14 ",O6)</f>
+      </c>
+      <c r="J129" s="22"/>
+      <c r="K129" s="22"/>
+      <c r="L129" s="22"/>
+      <c r="M129" s="22"/>
+      <c r="N129" s="22"/>
+      <c r="O129" s="19" t="str">
+        <f>'data'!$B$50</f>
+      </c>
+    </row>
+    <row r="131">
+      <c r="F131" t="s">
         <v>304</v>
       </c>
-      <c r="G118" s="23"/>
-      <c r="N118" t="s">
+      <c r="G131" s="23"/>
+      <c r="N131" t="s">
         <v>304</v>
       </c>
-      <c r="O118" s="23"/>
-    </row>
-    <row r="119">
-      <c r="F119" t="s">
+      <c r="O131" s="23"/>
+    </row>
+    <row r="132">
+      <c r="F132" t="s">
         <v>305</v>
       </c>
-      <c r="G119" s="23"/>
-      <c r="N119" t="s">
+      <c r="G132" s="23"/>
+      <c r="N132" t="s">
         <v>305</v>
       </c>
-      <c r="O119" s="23"/>
-    </row>
-    <row r="122">
-      <c r="A122" s="11" t="s">
-        <v>335</v>
-      </c>
-      <c r="B122" s="11"/>
-      <c r="C122" s="11"/>
-      <c r="D122" s="11"/>
-      <c r="E122" s="11"/>
-      <c r="F122" s="11"/>
-      <c r="G122" s="11"/>
-      <c r="I122" s="11" t="s">
-        <v>336</v>
-      </c>
-      <c r="J122" s="11"/>
-      <c r="K122" s="11"/>
-      <c r="L122" s="11"/>
-      <c r="M122" s="11"/>
-      <c r="N122" s="11"/>
-      <c r="O122" s="11"/>
-    </row>
-    <row r="123">
-      <c r="A123" s="21" t="s">
-        <v>301</v>
-      </c>
-      <c r="D123" s="19" t="s">
-        <v>302</v>
-      </c>
-      <c r="G123" s="20" t="s">
-        <v>303</v>
-      </c>
-      <c r="I123" s="21" t="s">
-        <v>301</v>
-      </c>
-      <c r="L123" s="19" t="s">
-        <v>302</v>
-      </c>
-      <c r="O123" s="20" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="19" t="str">
-        <f>'data'!$B$47</f>
-      </c>
-      <c r="B124" s="22"/>
-      <c r="C124" s="22"/>
-      <c r="D124" s="22"/>
-      <c r="E124" s="22"/>
-      <c r="F124" s="22"/>
-      <c r="G124" s="19" t="str">
-        <f>'data'!$B$46</f>
-      </c>
-      <c r="I124" s="19" t="str">
-        <f>'data'!$B$93</f>
-      </c>
-      <c r="J124" s="22"/>
-      <c r="K124" s="22"/>
-      <c r="L124" s="22"/>
-      <c r="M124" s="22"/>
-      <c r="N124" s="22"/>
-      <c r="O124" s="19" t="str">
-        <f>'data'!$B$92</f>
-      </c>
-    </row>
-    <row r="126">
-      <c r="F126" t="s">
-        <v>304</v>
-      </c>
-      <c r="G126" s="23"/>
-      <c r="N126" t="s">
-        <v>304</v>
-      </c>
-      <c r="O126" s="23"/>
-    </row>
-    <row r="127">
-      <c r="F127" t="s">
-        <v>305</v>
-      </c>
-      <c r="G127" s="23"/>
-      <c r="N127" t="s">
-        <v>305</v>
-      </c>
-      <c r="O127" s="23"/>
+      <c r="O132" s="23"/>
     </row>
     <row r="135">
       <c r="A135" s="11" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B135" s="11"/>
       <c r="C135" s="11"/>
@@ -7242,7 +7223,7 @@
       <c r="F135" s="11"/>
       <c r="G135" s="11"/>
       <c r="I135" s="11" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="J135" s="11"/>
       <c r="K135" s="11"/>
@@ -7281,10 +7262,10 @@
       <c r="E137" s="22"/>
       <c r="F137" s="22"/>
       <c r="G137" s="19" t="str">
-        <f>'data'!$B$5</f>
+        <f>'data'!$B$8</f>
       </c>
       <c r="I137" s="19" t="str">
-        <f>CONCATENATE("M 18 ",O14)</f>
+        <f>CONCATENATE("M 15 ",O14)</f>
       </c>
       <c r="J137" s="22"/>
       <c r="K137" s="22"/>
@@ -7292,7 +7273,7 @@
       <c r="M137" s="22"/>
       <c r="N137" s="22"/>
       <c r="O137" s="19" t="str">
-        <f>'data'!$B$50</f>
+        <f>'data'!$B$53</f>
       </c>
     </row>
     <row r="139">
@@ -7317,7 +7298,7 @@
     </row>
     <row r="143">
       <c r="A143" s="11" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B143" s="11"/>
       <c r="C143" s="11"/>
@@ -7326,7 +7307,7 @@
       <c r="F143" s="11"/>
       <c r="G143" s="11"/>
       <c r="I143" s="11" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J143" s="11"/>
       <c r="K143" s="11"/>
@@ -7365,10 +7346,10 @@
       <c r="E145" s="22"/>
       <c r="F145" s="22"/>
       <c r="G145" s="19" t="str">
-        <f>'data'!$B$8</f>
+        <f>'data'!$B$89</f>
       </c>
       <c r="I145" s="19" t="str">
-        <f>CONCATENATE("M 19 ",O22)</f>
+        <f>CONCATENATE("M 16 ",O22)</f>
       </c>
       <c r="J145" s="22"/>
       <c r="K145" s="22"/>
@@ -7376,7 +7357,7 @@
       <c r="M145" s="22"/>
       <c r="N145" s="22"/>
       <c r="O145" s="19" t="str">
-        <f>'data'!$B$53</f>
+        <f>'data'!$B$56</f>
       </c>
     </row>
     <row r="147">
@@ -7401,7 +7382,7 @@
     </row>
     <row r="151">
       <c r="A151" s="11" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B151" s="11"/>
       <c r="C151" s="11"/>
@@ -7410,7 +7391,7 @@
       <c r="F151" s="11"/>
       <c r="G151" s="11"/>
       <c r="I151" s="11" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="J151" s="11"/>
       <c r="K151" s="11"/>
@@ -7441,7 +7422,7 @@
     </row>
     <row r="153">
       <c r="A153" s="19" t="str">
-        <f>CONCATENATE("M 4 ",G30)</f>
+        <f>'data'!$B$15</f>
       </c>
       <c r="B153" s="22"/>
       <c r="C153" s="22"/>
@@ -7449,10 +7430,10 @@
       <c r="E153" s="22"/>
       <c r="F153" s="22"/>
       <c r="G153" s="19" t="str">
-        <f>'data'!$B$89</f>
+        <f>'data'!$B$14</f>
       </c>
       <c r="I153" s="19" t="str">
-        <f>CONCATENATE("M 20 ",O30)</f>
+        <f>CONCATENATE("M 17 ",O30)</f>
       </c>
       <c r="J153" s="22"/>
       <c r="K153" s="22"/>
@@ -7460,7 +7441,7 @@
       <c r="M153" s="22"/>
       <c r="N153" s="22"/>
       <c r="O153" s="19" t="str">
-        <f>'data'!$B$56</f>
+        <f>'data'!$B$79</f>
       </c>
     </row>
     <row r="155">
@@ -7485,7 +7466,7 @@
     </row>
     <row r="159">
       <c r="A159" s="11" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B159" s="11"/>
       <c r="C159" s="11"/>
@@ -7494,7 +7475,7 @@
       <c r="F159" s="11"/>
       <c r="G159" s="11"/>
       <c r="I159" s="11" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="J159" s="11"/>
       <c r="K159" s="11"/>
@@ -7525,7 +7506,7 @@
     </row>
     <row r="161">
       <c r="A161" s="19" t="str">
-        <f>CONCATENATE("M 6 ",G46)</f>
+        <f>CONCATENATE("M 4 ",G30)</f>
       </c>
       <c r="B161" s="22"/>
       <c r="C161" s="22"/>
@@ -7536,7 +7517,7 @@
         <f>'data'!$B$16</f>
       </c>
       <c r="I161" s="19" t="str">
-        <f>CONCATENATE("M 21 ",O38)</f>
+        <f>CONCATENATE("M 18 ",O38)</f>
       </c>
       <c r="J161" s="22"/>
       <c r="K161" s="22"/>
@@ -7544,7 +7525,7 @@
       <c r="M161" s="22"/>
       <c r="N161" s="22"/>
       <c r="O161" s="19" t="str">
-        <f>'data'!$B$79</f>
+        <f>'data'!$B$62</f>
       </c>
     </row>
     <row r="163">
@@ -7569,7 +7550,7 @@
     </row>
     <row r="167">
       <c r="A167" s="11" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B167" s="11"/>
       <c r="C167" s="11"/>
@@ -7578,7 +7559,7 @@
       <c r="F167" s="11"/>
       <c r="G167" s="11"/>
       <c r="I167" s="11" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="J167" s="11"/>
       <c r="K167" s="11"/>
@@ -7609,7 +7590,7 @@
     </row>
     <row r="169">
       <c r="A169" s="19" t="str">
-        <f>CONCATENATE("M 7 ",G54)</f>
+        <f>CONCATENATE("M 5 ",G38)</f>
       </c>
       <c r="B169" s="22"/>
       <c r="C169" s="22"/>
@@ -7620,7 +7601,7 @@
         <f>'data'!$B$19</f>
       </c>
       <c r="I169" s="19" t="str">
-        <f>CONCATENATE("M 22 ",O46)</f>
+        <f>CONCATENATE("M 19 ",O46)</f>
       </c>
       <c r="J169" s="22"/>
       <c r="K169" s="22"/>
@@ -7628,7 +7609,7 @@
       <c r="M169" s="22"/>
       <c r="N169" s="22"/>
       <c r="O169" s="19" t="str">
-        <f>'data'!$B$62</f>
+        <f>'data'!$B$65</f>
       </c>
     </row>
     <row r="171">
@@ -7653,7 +7634,7 @@
     </row>
     <row r="175">
       <c r="A175" s="11" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B175" s="11"/>
       <c r="C175" s="11"/>
@@ -7662,7 +7643,7 @@
       <c r="F175" s="11"/>
       <c r="G175" s="11"/>
       <c r="I175" s="11" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="J175" s="11"/>
       <c r="K175" s="11"/>
@@ -7693,7 +7674,7 @@
     </row>
     <row r="177">
       <c r="A177" s="19" t="str">
-        <f>CONCATENATE("M 8 ",G62)</f>
+        <f>CONCATENATE("M 6 ",G46)</f>
       </c>
       <c r="B177" s="22"/>
       <c r="C177" s="22"/>
@@ -7704,7 +7685,7 @@
         <f>'data'!$B$22</f>
       </c>
       <c r="I177" s="19" t="str">
-        <f>CONCATENATE("M 23 ",O54)</f>
+        <f>CONCATENATE("M 20 ",O54)</f>
       </c>
       <c r="J177" s="22"/>
       <c r="K177" s="22"/>
@@ -7712,7 +7693,7 @@
       <c r="M177" s="22"/>
       <c r="N177" s="22"/>
       <c r="O177" s="19" t="str">
-        <f>'data'!$B$65</f>
+        <f>'data'!$B$68</f>
       </c>
     </row>
     <row r="179">
@@ -7737,7 +7718,7 @@
     </row>
     <row r="183">
       <c r="A183" s="11" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B183" s="11"/>
       <c r="C183" s="11"/>
@@ -7746,7 +7727,7 @@
       <c r="F183" s="11"/>
       <c r="G183" s="11"/>
       <c r="I183" s="11" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="J183" s="11"/>
       <c r="K183" s="11"/>
@@ -7777,7 +7758,7 @@
     </row>
     <row r="185">
       <c r="A185" s="19" t="str">
-        <f>CONCATENATE("M 10 ",G78)</f>
+        <f>'data'!$B$26</f>
       </c>
       <c r="B185" s="22"/>
       <c r="C185" s="22"/>
@@ -7785,10 +7766,10 @@
       <c r="E185" s="22"/>
       <c r="F185" s="22"/>
       <c r="G185" s="19" t="str">
-        <f>'data'!$B$31</f>
+        <f>'data'!$B$25</f>
       </c>
       <c r="I185" s="19" t="str">
-        <f>CONCATENATE("M 24 ",O62)</f>
+        <f>'data'!$B$72</f>
       </c>
       <c r="J185" s="22"/>
       <c r="K185" s="22"/>
@@ -7796,7 +7777,7 @@
       <c r="M185" s="22"/>
       <c r="N185" s="22"/>
       <c r="O185" s="19" t="str">
-        <f>'data'!$B$68</f>
+        <f>'data'!$B$71</f>
       </c>
     </row>
     <row r="187">
@@ -7821,7 +7802,7 @@
     </row>
     <row r="191">
       <c r="A191" s="11" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B191" s="11"/>
       <c r="C191" s="11"/>
@@ -7830,7 +7811,7 @@
       <c r="F191" s="11"/>
       <c r="G191" s="11"/>
       <c r="I191" s="11" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="J191" s="11"/>
       <c r="K191" s="11"/>
@@ -7861,7 +7842,7 @@
     </row>
     <row r="193">
       <c r="A193" s="19" t="str">
-        <f>CONCATENATE("M 11 ",G86)</f>
+        <f>CONCATENATE("M 7 ",G54)</f>
       </c>
       <c r="B193" s="22"/>
       <c r="C193" s="22"/>
@@ -7869,10 +7850,10 @@
       <c r="E193" s="22"/>
       <c r="F193" s="22"/>
       <c r="G193" s="19" t="str">
-        <f>'data'!$B$67</f>
+        <f>'data'!$B$31</f>
       </c>
       <c r="I193" s="19" t="str">
-        <f>CONCATENATE("M 26 ",O78)</f>
+        <f>CONCATENATE("M 21 ",O62)</f>
       </c>
       <c r="J193" s="22"/>
       <c r="K193" s="22"/>
@@ -7905,7 +7886,7 @@
     </row>
     <row r="199">
       <c r="A199" s="11" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B199" s="11"/>
       <c r="C199" s="11"/>
@@ -7914,7 +7895,7 @@
       <c r="F199" s="11"/>
       <c r="G199" s="11"/>
       <c r="I199" s="11" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="J199" s="11"/>
       <c r="K199" s="11"/>
@@ -7945,7 +7926,7 @@
     </row>
     <row r="201">
       <c r="A201" s="19" t="str">
-        <f>CONCATENATE("M 12 ",G94)</f>
+        <f>CONCATENATE("M 8 ",G62)</f>
       </c>
       <c r="B201" s="22"/>
       <c r="C201" s="22"/>
@@ -7953,10 +7934,10 @@
       <c r="E201" s="22"/>
       <c r="F201" s="22"/>
       <c r="G201" s="19" t="str">
-        <f>'data'!$B$78</f>
+        <f>'data'!$B$67</f>
       </c>
       <c r="I201" s="19" t="str">
-        <f>CONCATENATE("M 27 ",O86)</f>
+        <f>CONCATENATE("M 22 ",O70)</f>
       </c>
       <c r="J201" s="22"/>
       <c r="K201" s="22"/>
@@ -7989,7 +7970,7 @@
     </row>
     <row r="207">
       <c r="A207" s="11" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B207" s="11"/>
       <c r="C207" s="11"/>
@@ -7998,7 +7979,7 @@
       <c r="F207" s="11"/>
       <c r="G207" s="11"/>
       <c r="I207" s="11" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="J207" s="11"/>
       <c r="K207" s="11"/>
@@ -8029,7 +8010,7 @@
     </row>
     <row r="209">
       <c r="A209" s="19" t="str">
-        <f>CONCATENATE("M 13 ",G102)</f>
+        <f>CONCATENATE("M 9 ",G70)</f>
       </c>
       <c r="B209" s="22"/>
       <c r="C209" s="22"/>
@@ -8037,10 +8018,10 @@
       <c r="E209" s="22"/>
       <c r="F209" s="22"/>
       <c r="G209" s="19" t="str">
-        <f>'data'!$B$57</f>
+        <f>'data'!$B$78</f>
       </c>
       <c r="I209" s="19" t="str">
-        <f>CONCATENATE("M 28 ",O94)</f>
+        <f>CONCATENATE("M 23 ",O78)</f>
       </c>
       <c r="J209" s="22"/>
       <c r="K209" s="22"/>
@@ -8073,7 +8054,7 @@
     </row>
     <row r="215">
       <c r="A215" s="11" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B215" s="11"/>
       <c r="C215" s="11"/>
@@ -8082,7 +8063,7 @@
       <c r="F215" s="11"/>
       <c r="G215" s="11"/>
       <c r="I215" s="11" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="J215" s="11"/>
       <c r="K215" s="11"/>
@@ -8113,7 +8094,7 @@
     </row>
     <row r="217">
       <c r="A217" s="19" t="str">
-        <f>CONCATENATE("M 14 ",G110)</f>
+        <f>CONCATENATE("M 10 ",G78)</f>
       </c>
       <c r="B217" s="22"/>
       <c r="C217" s="22"/>
@@ -8121,10 +8102,10 @@
       <c r="E217" s="22"/>
       <c r="F217" s="22"/>
       <c r="G217" s="19" t="str">
-        <f>'data'!$B$39</f>
+        <f>'data'!$B$57</f>
       </c>
       <c r="I217" s="19" t="str">
-        <f>CONCATENATE("M 29 ",O102)</f>
+        <f>CONCATENATE("M 24 ",O86)</f>
       </c>
       <c r="J217" s="22"/>
       <c r="K217" s="22"/>
@@ -8157,7 +8138,7 @@
     </row>
     <row r="223">
       <c r="A223" s="11" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B223" s="11"/>
       <c r="C223" s="11"/>
@@ -8166,7 +8147,7 @@
       <c r="F223" s="11"/>
       <c r="G223" s="11"/>
       <c r="I223" s="11" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="J223" s="11"/>
       <c r="K223" s="11"/>
@@ -8197,7 +8178,7 @@
     </row>
     <row r="225">
       <c r="A225" s="19" t="str">
-        <f>CONCATENATE("M 15 ",G118)</f>
+        <f>CONCATENATE("M 11 ",G86)</f>
       </c>
       <c r="B225" s="22"/>
       <c r="C225" s="22"/>
@@ -8205,10 +8186,10 @@
       <c r="E225" s="22"/>
       <c r="F225" s="22"/>
       <c r="G225" s="19" t="str">
-        <f>'data'!$B$42</f>
+        <f>'data'!$B$39</f>
       </c>
       <c r="I225" s="19" t="str">
-        <f>CONCATENATE("M 30 ",O110)</f>
+        <f>CONCATENATE("M 25 ",O94)</f>
       </c>
       <c r="J225" s="22"/>
       <c r="K225" s="22"/>
@@ -8241,7 +8222,7 @@
     </row>
     <row r="231">
       <c r="A231" s="11" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B231" s="11"/>
       <c r="C231" s="11"/>
@@ -8250,7 +8231,7 @@
       <c r="F231" s="11"/>
       <c r="G231" s="11"/>
       <c r="I231" s="11" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="J231" s="11"/>
       <c r="K231" s="11"/>
@@ -8281,7 +8262,7 @@
     </row>
     <row r="233">
       <c r="A233" s="19" t="str">
-        <f>CONCATENATE("M 16 ",G126)</f>
+        <f>CONCATENATE("M 12 ",G94)</f>
       </c>
       <c r="B233" s="22"/>
       <c r="C233" s="22"/>
@@ -8289,10 +8270,10 @@
       <c r="E233" s="22"/>
       <c r="F233" s="22"/>
       <c r="G233" s="19" t="str">
-        <f>'data'!$B$45</f>
+        <f>'data'!$B$42</f>
       </c>
       <c r="I233" s="19" t="str">
-        <f>CONCATENATE("M 31 ",O118)</f>
+        <f>CONCATENATE("M 26 ",O102)</f>
       </c>
       <c r="J233" s="22"/>
       <c r="K233" s="22"/>
@@ -8324,6 +8305,15 @@
       <c r="O236" s="23"/>
     </row>
     <row r="239">
+      <c r="A239" s="11" t="s">
+        <v>362</v>
+      </c>
+      <c r="B239" s="11"/>
+      <c r="C239" s="11"/>
+      <c r="D239" s="11"/>
+      <c r="E239" s="11"/>
+      <c r="F239" s="11"/>
+      <c r="G239" s="11"/>
       <c r="I239" s="11" t="s">
         <v>363</v>
       </c>
@@ -8335,6 +8325,15 @@
       <c r="O239" s="11"/>
     </row>
     <row r="240">
+      <c r="A240" s="21" t="s">
+        <v>301</v>
+      </c>
+      <c r="D240" s="19" t="s">
+        <v>302</v>
+      </c>
+      <c r="G240" s="20" t="s">
+        <v>303</v>
+      </c>
       <c r="I240" s="21" t="s">
         <v>301</v>
       </c>
@@ -8346,8 +8345,19 @@
       </c>
     </row>
     <row r="241">
+      <c r="A241" s="19" t="str">
+        <f>CONCATENATE("M 13 ",G102)</f>
+      </c>
+      <c r="B241" s="22"/>
+      <c r="C241" s="22"/>
+      <c r="D241" s="22"/>
+      <c r="E241" s="22"/>
+      <c r="F241" s="22"/>
+      <c r="G241" s="19" t="str">
+        <f>'data'!$B$45</f>
+      </c>
       <c r="I241" s="19" t="str">
-        <f>CONCATENATE("M 32 ",O126)</f>
+        <f>CONCATENATE("M 27 ",O110)</f>
       </c>
       <c r="J241" s="22"/>
       <c r="K241" s="22"/>
@@ -8359,12 +8369,20 @@
       </c>
     </row>
     <row r="243">
+      <c r="F243" t="s">
+        <v>304</v>
+      </c>
+      <c r="G243" s="23"/>
       <c r="N243" t="s">
         <v>304</v>
       </c>
       <c r="O243" s="23"/>
     </row>
     <row r="244">
+      <c r="F244" t="s">
+        <v>305</v>
+      </c>
+      <c r="G244" s="23"/>
       <c r="N244" t="s">
         <v>305</v>
       </c>
@@ -8412,7 +8430,7 @@
     </row>
     <row r="254">
       <c r="A254" s="19" t="str">
-        <f>CONCATENATE("M 33 ",G139)</f>
+        <f>CONCATENATE("M 29 ",G131)</f>
       </c>
       <c r="B254" s="22"/>
       <c r="C254" s="22"/>
@@ -8420,10 +8438,10 @@
       <c r="E254" s="22"/>
       <c r="F254" s="22"/>
       <c r="G254" s="19" t="str">
-        <f>CONCATENATE("M 1 ",G6)</f>
+        <f>CONCATENATE("M 28 ",G123)</f>
       </c>
       <c r="I254" s="19" t="str">
-        <f>CONCATENATE("M 46 ",O139)</f>
+        <f>CONCATENATE("M 45 ",O131)</f>
       </c>
       <c r="J254" s="22"/>
       <c r="K254" s="22"/>
@@ -8431,7 +8449,7 @@
       <c r="M254" s="22"/>
       <c r="N254" s="22"/>
       <c r="O254" s="19" t="str">
-        <f>CONCATENATE("M 17 ",O6)</f>
+        <f>CONCATENATE("M 44 ",O123)</f>
       </c>
     </row>
     <row r="256">
@@ -8496,7 +8514,7 @@
     </row>
     <row r="262">
       <c r="A262" s="19" t="str">
-        <f>CONCATENATE("M 35 ",G155)</f>
+        <f>CONCATENATE("M 31 ",G147)</f>
       </c>
       <c r="B262" s="22"/>
       <c r="C262" s="22"/>
@@ -8504,10 +8522,10 @@
       <c r="E262" s="22"/>
       <c r="F262" s="22"/>
       <c r="G262" s="19" t="str">
-        <f>CONCATENATE("M 34 ",G147)</f>
+        <f>CONCATENATE("M 30 ",G139)</f>
       </c>
       <c r="I262" s="19" t="str">
-        <f>CONCATENATE("M 48 ",O155)</f>
+        <f>CONCATENATE("M 47 ",O147)</f>
       </c>
       <c r="J262" s="22"/>
       <c r="K262" s="22"/>
@@ -8515,7 +8533,7 @@
       <c r="M262" s="22"/>
       <c r="N262" s="22"/>
       <c r="O262" s="19" t="str">
-        <f>CONCATENATE("M 47 ",O147)</f>
+        <f>CONCATENATE("M 46 ",O139)</f>
       </c>
     </row>
     <row r="264">
@@ -8580,7 +8598,7 @@
     </row>
     <row r="270">
       <c r="A270" s="19" t="str">
-        <f>CONCATENATE("M 36 ",G163)</f>
+        <f>CONCATENATE("M 33 ",G163)</f>
       </c>
       <c r="B270" s="22"/>
       <c r="C270" s="22"/>
@@ -8588,10 +8606,10 @@
       <c r="E270" s="22"/>
       <c r="F270" s="22"/>
       <c r="G270" s="19" t="str">
-        <f>CONCATENATE("M 5 ",G38)</f>
+        <f>CONCATENATE("M 32 ",G155)</f>
       </c>
       <c r="I270" s="19" t="str">
-        <f>CONCATENATE("M 50 ",O171)</f>
+        <f>CONCATENATE("M 49 ",O163)</f>
       </c>
       <c r="J270" s="22"/>
       <c r="K270" s="22"/>
@@ -8599,7 +8617,7 @@
       <c r="M270" s="22"/>
       <c r="N270" s="22"/>
       <c r="O270" s="19" t="str">
-        <f>CONCATENATE("M 49 ",O163)</f>
+        <f>CONCATENATE("M 48 ",O155)</f>
       </c>
     </row>
     <row r="272">
@@ -8664,7 +8682,7 @@
     </row>
     <row r="278">
       <c r="A278" s="19" t="str">
-        <f>CONCATENATE("M 38 ",G179)</f>
+        <f>CONCATENATE("M 35 ",G179)</f>
       </c>
       <c r="B278" s="22"/>
       <c r="C278" s="22"/>
@@ -8672,10 +8690,10 @@
       <c r="E278" s="22"/>
       <c r="F278" s="22"/>
       <c r="G278" s="19" t="str">
-        <f>CONCATENATE("M 37 ",G171)</f>
+        <f>CONCATENATE("M 34 ",G171)</f>
       </c>
       <c r="I278" s="19" t="str">
-        <f>CONCATENATE("M 52 ",O187)</f>
+        <f>CONCATENATE("M 51 ",O179)</f>
       </c>
       <c r="J278" s="22"/>
       <c r="K278" s="22"/>
@@ -8683,7 +8701,7 @@
       <c r="M278" s="22"/>
       <c r="N278" s="22"/>
       <c r="O278" s="19" t="str">
-        <f>CONCATENATE("M 51 ",O179)</f>
+        <f>CONCATENATE("M 50 ",O171)</f>
       </c>
     </row>
     <row r="280">
@@ -8748,7 +8766,7 @@
     </row>
     <row r="286">
       <c r="A286" s="19" t="str">
-        <f>CONCATENATE("M 39 ",G187)</f>
+        <f>CONCATENATE("M 37 ",G195)</f>
       </c>
       <c r="B286" s="22"/>
       <c r="C286" s="22"/>
@@ -8756,7 +8774,7 @@
       <c r="E286" s="22"/>
       <c r="F286" s="22"/>
       <c r="G286" s="19" t="str">
-        <f>CONCATENATE("M 9 ",G70)</f>
+        <f>CONCATENATE("M 36 ",G187)</f>
       </c>
       <c r="I286" s="19" t="str">
         <f>CONCATENATE("M 53 ",O195)</f>
@@ -8767,7 +8785,7 @@
       <c r="M286" s="22"/>
       <c r="N286" s="22"/>
       <c r="O286" s="19" t="str">
-        <f>CONCATENATE("M 25 ",O70)</f>
+        <f>CONCATENATE("M 52 ",O187)</f>
       </c>
     </row>
     <row r="288">
@@ -8832,7 +8850,7 @@
     </row>
     <row r="294">
       <c r="A294" s="19" t="str">
-        <f>CONCATENATE("M 41 ",G203)</f>
+        <f>CONCATENATE("M 39 ",G211)</f>
       </c>
       <c r="B294" s="22"/>
       <c r="C294" s="22"/>
@@ -8840,7 +8858,7 @@
       <c r="E294" s="22"/>
       <c r="F294" s="22"/>
       <c r="G294" s="19" t="str">
-        <f>CONCATENATE("M 40 ",G195)</f>
+        <f>CONCATENATE("M 38 ",G203)</f>
       </c>
       <c r="I294" s="19" t="str">
         <f>CONCATENATE("M 55 ",O211)</f>
@@ -8916,7 +8934,7 @@
     </row>
     <row r="302">
       <c r="A302" s="19" t="str">
-        <f>CONCATENATE("M 43 ",G219)</f>
+        <f>CONCATENATE("M 41 ",G227)</f>
       </c>
       <c r="B302" s="22"/>
       <c r="C302" s="22"/>
@@ -8924,7 +8942,7 @@
       <c r="E302" s="22"/>
       <c r="F302" s="22"/>
       <c r="G302" s="19" t="str">
-        <f>CONCATENATE("M 42 ",G211)</f>
+        <f>CONCATENATE("M 40 ",G219)</f>
       </c>
       <c r="I302" s="19" t="str">
         <f>CONCATENATE("M 57 ",O227)</f>
@@ -9000,7 +9018,7 @@
     </row>
     <row r="310">
       <c r="A310" s="19" t="str">
-        <f>CONCATENATE("M 45 ",G235)</f>
+        <f>CONCATENATE("M 43 ",G243)</f>
       </c>
       <c r="B310" s="22"/>
       <c r="C310" s="22"/>
@@ -9008,7 +9026,7 @@
       <c r="E310" s="22"/>
       <c r="F310" s="22"/>
       <c r="G310" s="19" t="str">
-        <f>CONCATENATE("M 44 ",G227)</f>
+        <f>CONCATENATE("M 42 ",G235)</f>
       </c>
       <c r="I310" s="19" t="str">
         <f>CONCATENATE("M 59 ",O243)</f>
@@ -9708,12 +9726,11 @@
     <mergeCell ref="I90:O90"/>
     <mergeCell ref="A98:G98"/>
     <mergeCell ref="I98:O98"/>
-    <mergeCell ref="A106:G106"/>
     <mergeCell ref="I106:O106"/>
-    <mergeCell ref="A114:G114"/>
-    <mergeCell ref="I114:O114"/>
-    <mergeCell ref="A122:G122"/>
-    <mergeCell ref="I122:O122"/>
+    <mergeCell ref="A119:G119"/>
+    <mergeCell ref="I119:O119"/>
+    <mergeCell ref="A127:G127"/>
+    <mergeCell ref="I127:O127"/>
     <mergeCell ref="A135:G135"/>
     <mergeCell ref="I135:O135"/>
     <mergeCell ref="A143:G143"/>
@@ -9740,6 +9757,7 @@
     <mergeCell ref="I223:O223"/>
     <mergeCell ref="A231:G231"/>
     <mergeCell ref="I231:O231"/>
+    <mergeCell ref="A239:G239"/>
     <mergeCell ref="I239:O239"/>
     <mergeCell ref="A252:G252"/>
     <mergeCell ref="I252:O252"/>
@@ -9778,7 +9796,7 @@
   <rowBreaks count="9" manualBreakCount="9">
     <brk id="41" max="16383" man="true"/>
     <brk id="81" max="16383" man="true"/>
-    <brk id="121" max="16383" man="true"/>
+    <brk id="118" max="16383" man="true"/>
     <brk id="158" max="16383" man="true"/>
     <brk id="198" max="16383" man="true"/>
     <brk id="238" max="16383" man="true"/>
@@ -9821,29 +9839,35 @@
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
     </row>
-    <row r="5">
-      <c r="C5" s="16" t="s">
+    <row r="6">
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6">
-      <c r="D6" s="14"/>
-      <c r="E6" s="13">
-        <v>1</v>
-      </c>
-    </row>
     <row r="7">
-      <c r="C7" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="12"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="12"/>
+    </row>
+    <row r="8">
+      <c r="G8" s="13">
+        <v>28</v>
+      </c>
     </row>
     <row r="9">
+      <c r="G9" s="12"/>
       <c r="H9" s="14"/>
       <c r="I9" s="12"/>
     </row>
     <row r="10">
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="15"/>
+      <c r="G10" s="12"/>
       <c r="I10" s="12"/>
     </row>
     <row r="11">
@@ -9876,7 +9900,7 @@
     </row>
     <row r="16">
       <c r="G16" s="13">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="H16" s="15"/>
       <c r="I16" s="12"/>
@@ -9892,7 +9916,7 @@
     <row r="18">
       <c r="D18" s="14"/>
       <c r="E18" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18" s="15"/>
       <c r="G18" s="12"/>
@@ -9929,7 +9953,7 @@
     </row>
     <row r="24">
       <c r="G24" s="13">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="K24" s="12"/>
     </row>
@@ -9945,7 +9969,7 @@
     <row r="26">
       <c r="D26" s="14"/>
       <c r="E26" s="13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26" s="15"/>
       <c r="G26" s="12"/>
@@ -9986,7 +10010,7 @@
     </row>
     <row r="32">
       <c r="G32" s="13">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H32" s="15"/>
       <c r="I32" s="12"/>
@@ -10000,7 +10024,7 @@
     <row r="34">
       <c r="D34" s="14"/>
       <c r="E34" s="13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F34" s="15"/>
       <c r="G34" s="12"/>
@@ -10051,29 +10075,35 @@
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
     </row>
-    <row r="5">
-      <c r="C5" s="16" t="s">
+    <row r="6">
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="6">
-      <c r="D6" s="14"/>
-      <c r="E6" s="13">
-        <v>5</v>
-      </c>
-    </row>
     <row r="7">
-      <c r="C7" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="12"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="12"/>
+    </row>
+    <row r="8">
+      <c r="G8" s="13">
+        <v>32</v>
+      </c>
     </row>
     <row r="9">
+      <c r="G9" s="12"/>
       <c r="H9" s="14"/>
       <c r="I9" s="12"/>
     </row>
     <row r="10">
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" s="15"/>
+      <c r="G10" s="12"/>
       <c r="I10" s="12"/>
     </row>
     <row r="11">
@@ -10106,7 +10136,7 @@
     </row>
     <row r="16">
       <c r="G16" s="13">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="H16" s="15"/>
       <c r="I16" s="12"/>
@@ -10122,7 +10152,7 @@
     <row r="18">
       <c r="D18" s="14"/>
       <c r="E18" s="13">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F18" s="15"/>
       <c r="G18" s="12"/>
@@ -10159,7 +10189,7 @@
     </row>
     <row r="24">
       <c r="G24" s="13">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K24" s="12"/>
     </row>
@@ -10175,7 +10205,7 @@
     <row r="26">
       <c r="D26" s="14"/>
       <c r="E26" s="13">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F26" s="15"/>
       <c r="G26" s="12"/>
@@ -10216,7 +10246,7 @@
     </row>
     <row r="32">
       <c r="G32" s="13">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="H32" s="15"/>
       <c r="I32" s="12"/>
@@ -10230,7 +10260,7 @@
     <row r="34">
       <c r="D34" s="14"/>
       <c r="E34" s="13">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F34" s="15"/>
       <c r="G34" s="12"/>

</xml_diff>

<commit_message>
chore(bc-dhas): regenerate the knockout example workbooks
7c056ba9 keyed knockout entrants by entrant rather than by name, so two
entrants who share a name (or a zekken) each keep their own data row. The
committed medium and large examples predate it: their Elimination Matches
sheet pointed some entrants' slots at a namesake's row, so a row was
referenced twice and another not at all. Regenerated with make examples,
every entrant is now referenced exactly once. The small example has no
namesakes and is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knockout-example-large-seeded.xlsx
+++ b/knockout-example-large-seeded.xlsx
@@ -5947,7 +5947,7 @@
     </row>
     <row r="4">
       <c r="A4" s="19" t="str">
-        <f>'data'!$B$80</f>
+        <f>'data'!$B$7</f>
       </c>
       <c r="B4" s="22"/>
       <c r="C4" s="22"/>
@@ -6039,7 +6039,7 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
       <c r="G12" s="19" t="str">
-        <f>'data'!$B$87</f>
+        <f>'data'!$B$9</f>
       </c>
       <c r="I12" s="19" t="str">
         <f>'data'!$B$55</f>
@@ -6123,7 +6123,7 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
       <c r="G20" s="19" t="str">
-        <f>'data'!$B$90</f>
+        <f>'data'!$B$12</f>
       </c>
       <c r="I20" s="19" t="str">
         <f>'data'!$B$58</f>
@@ -6470,7 +6470,7 @@
       <c r="M52" s="22"/>
       <c r="N52" s="22"/>
       <c r="O52" s="19" t="str">
-        <f>'data'!$B$73</f>
+        <f>'data'!$B$69</f>
       </c>
     </row>
     <row r="54">
@@ -6535,7 +6535,7 @@
     </row>
     <row r="60">
       <c r="A60" s="19" t="str">
-        <f>'data'!$B$55</f>
+        <f>'data'!$B$32</f>
       </c>
       <c r="B60" s="22"/>
       <c r="C60" s="22"/>
@@ -6627,7 +6627,7 @@
       <c r="E68" s="22"/>
       <c r="F68" s="22"/>
       <c r="G68" s="19" t="str">
-        <f>'data'!$B$56</f>
+        <f>'data'!$B$34</f>
       </c>
       <c r="I68" s="19" t="str">
         <f>'data'!$B$78</f>
@@ -6703,7 +6703,7 @@
     </row>
     <row r="76">
       <c r="A76" s="19" t="str">
-        <f>'data'!$B$70</f>
+        <f>'data'!$B$38</f>
       </c>
       <c r="B76" s="22"/>
       <c r="C76" s="22"/>
@@ -6711,7 +6711,7 @@
       <c r="E76" s="22"/>
       <c r="F76" s="22"/>
       <c r="G76" s="19" t="str">
-        <f>'data'!$B$53</f>
+        <f>'data'!$B$37</f>
       </c>
       <c r="I76" s="19" t="str">
         <f>'data'!$B$81</f>
@@ -6798,7 +6798,7 @@
         <f>'data'!$B$40</f>
       </c>
       <c r="I84" s="19" t="str">
-        <f>'data'!$B$93</f>
+        <f>'data'!$B$84</f>
       </c>
       <c r="J84" s="22"/>
       <c r="K84" s="22"/>
@@ -7094,7 +7094,7 @@
       <c r="E121" s="22"/>
       <c r="F121" s="22"/>
       <c r="G121" s="19" t="str">
-        <f>'data'!$B$60</f>
+        <f>'data'!$B$3</f>
       </c>
       <c r="I121" s="19" t="str">
         <f>'data'!$B$49</f>
@@ -7346,7 +7346,7 @@
       <c r="E145" s="22"/>
       <c r="F145" s="22"/>
       <c r="G145" s="19" t="str">
-        <f>'data'!$B$89</f>
+        <f>'data'!$B$11</f>
       </c>
       <c r="I145" s="19" t="str">
         <f>CONCATENATE("M 16 ",O22)</f>
@@ -7441,7 +7441,7 @@
       <c r="M153" s="22"/>
       <c r="N153" s="22"/>
       <c r="O153" s="19" t="str">
-        <f>'data'!$B$79</f>
+        <f>'data'!$B$59</f>
       </c>
     </row>
     <row r="155">
@@ -7850,7 +7850,7 @@
       <c r="E193" s="22"/>
       <c r="F193" s="22"/>
       <c r="G193" s="19" t="str">
-        <f>'data'!$B$31</f>
+        <f>'data'!$B$27</f>
       </c>
       <c r="I193" s="19" t="str">
         <f>CONCATENATE("M 21 ",O62)</f>
@@ -7934,7 +7934,7 @@
       <c r="E201" s="22"/>
       <c r="F201" s="22"/>
       <c r="G201" s="19" t="str">
-        <f>'data'!$B$67</f>
+        <f>'data'!$B$30</f>
       </c>
       <c r="I201" s="19" t="str">
         <f>CONCATENATE("M 22 ",O70)</f>
@@ -8018,7 +8018,7 @@
       <c r="E209" s="22"/>
       <c r="F209" s="22"/>
       <c r="G209" s="19" t="str">
-        <f>'data'!$B$78</f>
+        <f>'data'!$B$33</f>
       </c>
       <c r="I209" s="19" t="str">
         <f>CONCATENATE("M 23 ",O78)</f>
@@ -8102,7 +8102,7 @@
       <c r="E217" s="22"/>
       <c r="F217" s="22"/>
       <c r="G217" s="19" t="str">
-        <f>'data'!$B$57</f>
+        <f>'data'!$B$36</f>
       </c>
       <c r="I217" s="19" t="str">
         <f>CONCATENATE("M 24 ",O86)</f>

</xml_diff>

<commit_message>
build(deps): pin excelize to the master commit that fixes its 15 advisories
CI's validate job fails its Anchore image scan on main and on this PR
("vulnerabilities with level 'medium' or higher"). The only matches are
fifteen GHSA advisories against github.com/xuri/excelize/v2 v2.11.0, each
fixed only on excelize's master: no release after v2.11.0 exists yet. The
repo owner chose to pin that master commit here
(v2.11.1-0.20261010030226-066c84b8f7de, which brings github.com/xuri/efp
v0.0.2 with it); a grype scan of the rebuilt binary finds nothing.

The example workbooks are regenerated (make examples): the new excelize
writes each font's properties in a different order and a cell's number to
15 significant digits (Excel's own precision). Every cell value, formula,
style, page break and sheet is otherwise identical in all 17, checked by
comparing their XML with the numbers normalised.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knockout-example-large-seeded.xlsx
+++ b/knockout-example-large-seeded.xlsx
@@ -1257,79 +1257,79 @@
   </numFmts>
   <fonts count="11">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="12"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color rgb="FF000000"/>
-      <sz val="12"/>
     </font>
     <font>
+      <b val="1"/>
+      <u val="single"/>
+      <sz val="16"/>
+      <color/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color/>
-      <sz val="16"/>
-      <u val="single"/>
     </font>
     <font>
+      <b val="1"/>
+      <u val="single"/>
+      <sz val="12"/>
+      <color/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color/>
-      <sz val="12"/>
-      <u val="single"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color/>
-      <sz val="12"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="28"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="28"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="72"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="72"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="100"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="100"/>
     </font>
     <font>
+      <sz val="110"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color rgb="FF000000"/>
-      <sz val="110"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
     </font>
   </fonts>
   <fills count="5">
@@ -5639,16 +5639,16 @@
         <v>0</v>
       </c>
       <c r="D2" s="3">
-        <v>0.0020833333333333333</v>
+        <v>0.00208333333333333</v>
       </c>
       <c r="E2" s="3" t="str">
         <f>(A2*B2*C2*D2)</f>
       </c>
       <c r="F2" s="3">
-        <v>0.00034722222222222224</v>
+        <v>0.000347222222222222</v>
       </c>
       <c r="G2" s="3">
-        <v>0.020833333333333332</v>
+        <v>0.0208333333333333</v>
       </c>
       <c r="H2" s="24" t="str">
         <f>C2*I2+J2</f>
@@ -5665,16 +5665,16 @@
         <v>0</v>
       </c>
       <c r="D3" s="3">
-        <v>0.0020833333333333333</v>
+        <v>0.00208333333333333</v>
       </c>
       <c r="E3" s="3" t="str">
         <f>(A3*B3*C3*D3)</f>
       </c>
       <c r="F3" s="3">
-        <v>0.00034722222222222224</v>
+        <v>0.000347222222222222</v>
       </c>
       <c r="G3" s="3">
-        <v>0.020833333333333332</v>
+        <v>0.0208333333333333</v>
       </c>
       <c r="H3" s="3" t="str">
         <f>E3+(A3*C3*F3)+G3</f>
@@ -5743,16 +5743,16 @@
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="3">
-        <v>0.002777777777777778</v>
+        <v>0.00277777777777777</v>
       </c>
       <c r="E8" s="3" t="str">
         <f>(A8*B8*D8)</f>
       </c>
       <c r="F8" s="3">
-        <v>0.00034722222222222224</v>
+        <v>0.000347222222222222</v>
       </c>
       <c r="G8" s="3">
-        <v>0.020833333333333332</v>
+        <v>0.0208333333333333</v>
       </c>
       <c r="H8" s="24" t="str">
         <f>E8+(A8*F8)+G8</f>

</xml_diff>